<commit_message>
placon-arminio-tavares: param. V2 Híbrido com briefing revisado + docs
Re-briefing completo vs V1 (14/04): Laje Convencional→Protendida, Padrão
Médio→Médio-Alto, Fachada Cerâmica→Textura, Tipologia 1-2 Dorm→Misto,
Pé-direito 3,00→2,88m, Banheiros 2→1. Dados físicos atualizados do
arquitetônico PL_R05: AC 4.077,29 m², UR 55, NP 16/NPT 14, vagas 59.
Pressurização confirmada "Não" pelo PCI (EEV natural, não EPE).

Grand Total V2: R$ 18,4M / RSM² R$ 4.519 (+52% vs V1). Gerenciamento
inflado (22% vs 8-10% típico) por combinação AC pequena + prazo 24m.
Documentado na justificativa como candidato a override manual via
aba INDICES Col C.

Entregáveis: xlsx param. + docx justificativa + docx memorial. V1
arquivado em _antigo-parametrico-v1/. Script novo gerar_docs_placon_v2.py
lê direto do xlsx (via lib formulas) pra refletir V2 real.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/base/pacotes/placon-arminio-tavares/parametrico-placon-arminio-tavares.xlsx
+++ b/base/pacotes/placon-arminio-tavares/parametrico-placon-arminio-tavares.xlsx
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>4089.72</v>
+        <v>4077.29</v>
       </c>
     </row>
     <row r="6">
@@ -3791,7 +3791,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Convencional</t>
+          <t>Protendida</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Médio-Alto</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Cerâmica</t>
+          <t>Textura</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>1-2 Dormitórios</t>
+          <t>Misto</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Padrão (3.00)</t>
+          <t>Baixo (2.80)</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">

</xml_diff>